<commit_message>
comments nach diskussion mit andreas und simon
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\UZ_carrier_board\Project Outputs for UltraZOhm_CarrierBoard\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\UZ_carrier_board\Using Trenz Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="353">
   <si>
     <t>Quantity</t>
   </si>
@@ -1001,26 +1001,109 @@
     <t>hinzufügen!</t>
   </si>
   <si>
-    <t xml:space="preserve">alternative: MF-PSMF010X-2 </t>
-  </si>
-  <si>
-    <t>alternative: 595-TXS0108ERGYR  (differs in package)</t>
-  </si>
-  <si>
     <t>0402 available</t>
   </si>
   <si>
-    <t xml:space="preserve"> bereits hinzugefügt</t>
+    <t xml:space="preserve"> bereits hinzugefügt - passst</t>
+  </si>
+  <si>
+    <t>alternative, nein, da 100V, evtl 100uF für 5V (C66), sonst hinzufügen</t>
+  </si>
+  <si>
+    <t>hinzufügen oder 0402 auch ok</t>
+  </si>
+  <si>
+    <t>750-CPDA10R3V3U-HF</t>
+  </si>
+  <si>
+    <t>CPDA10R3V3U-HF</t>
+  </si>
+  <si>
+    <t>MBR0520L</t>
+  </si>
+  <si>
+    <t>hinzufügen, kleiner und günstigere alternative, ~100mA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0603 ist Ok </t>
+  </si>
+  <si>
+    <t>alternative: MF-PSMF010X-2  super</t>
+  </si>
+  <si>
+    <t>hinzufügen</t>
+  </si>
+  <si>
+    <t>verhältnis muss bleiben, check data sheet for range, 0402 wäre ok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1% needed - no </t>
+  </si>
+  <si>
+    <t>RESCAV80P160X320X70-8N</t>
+  </si>
+  <si>
+    <t>22843 47R 4fach, auch ok</t>
+  </si>
+  <si>
+    <t>schaltplan anpassen repeat(2) anstatt 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0402 available - ok </t>
+  </si>
+  <si>
+    <t>DMP4015SSS-13</t>
+  </si>
+  <si>
+    <t>double-check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">non-automotive? </t>
+  </si>
+  <si>
+    <t>SiT8008BI-73-33S-4.000000E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">any or-gate </t>
+  </si>
+  <si>
+    <t>check to replace with U23?</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>SN74LVC1G17DCKR</t>
+  </si>
+  <si>
+    <t>TI alternative? Andreas sucht was raus</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MMSZ5242BT1G   ???</t>
+  </si>
+  <si>
+    <t>SMBJ36CA</t>
+  </si>
+  <si>
+    <t>CDSOT23-T24CAN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1040,7 +1123,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1074,11 +1157,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1093,8 +1186,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1376,7 +1484,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q44"/>
+  <dimension ref="A1:T44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.1796875" customWidth="1"/>
@@ -1385,7 +1493,8 @@
     <col min="4" max="4" width="18.1796875" customWidth="1"/>
     <col min="5" max="5" width="20.36328125" customWidth="1"/>
     <col min="6" max="6" width="13.26953125" customWidth="1"/>
-    <col min="7" max="9" width="12.36328125" customWidth="1"/>
+    <col min="7" max="7" width="45.36328125" customWidth="1"/>
+    <col min="8" max="9" width="12.36328125" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="9.453125" customWidth="1"/>
@@ -1394,9 +1503,10 @@
     <col min="15" max="15" width="9.90625" customWidth="1"/>
     <col min="16" max="16" width="16" customWidth="1"/>
     <col min="17" max="17" width="43.6328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="26.6328125" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="1" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" s="1" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1448,8 +1558,9 @@
       <c r="Q1" s="1" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="R1" s="6"/>
+    </row>
+    <row r="2" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>3</v>
       </c>
@@ -1492,11 +1603,14 @@
       <c r="P2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" s="10" t="s">
         <v>320</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="R2" s="7" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>6</v>
       </c>
@@ -1545,11 +1659,11 @@
       <c r="P3" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="10" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="116" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -1598,11 +1712,11 @@
       <c r="P4" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q4" s="10" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="116" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>5</v>
       </c>
@@ -1652,10 +1766,10 @@
         <v>47</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" ht="72.5" x14ac:dyDescent="0.35">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>8</v>
       </c>
@@ -1704,8 +1818,17 @@
       <c r="P6" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+      <c r="Q6" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="R6" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="S6" s="9" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>1</v>
       </c>
@@ -1754,8 +1877,11 @@
       <c r="P7" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>1</v>
       </c>
@@ -1796,8 +1922,11 @@
       <c r="P8" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+      <c r="Q8" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>2</v>
       </c>
@@ -1846,8 +1975,14 @@
       <c r="P9" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" ht="116" x14ac:dyDescent="0.35">
+      <c r="Q9" t="s">
+        <v>352</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -1888,8 +2023,11 @@
       <c r="P10" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" ht="87" x14ac:dyDescent="0.35">
+      <c r="Q10" s="10" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>1</v>
       </c>
@@ -1938,7 +2076,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -1985,8 +2123,11 @@
       <c r="P12" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="Q12" s="5" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="58" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>1</v>
       </c>
@@ -2027,8 +2168,11 @@
       <c r="P13" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" ht="87" x14ac:dyDescent="0.35">
+      <c r="Q13" s="10" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="58" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>8</v>
       </c>
@@ -2069,11 +2213,11 @@
       <c r="P14" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q14" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" ht="174" x14ac:dyDescent="0.35">
+      <c r="Q14" s="10" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="58" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>3</v>
       </c>
@@ -2114,8 +2258,11 @@
       <c r="P15" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+      <c r="Q15" s="10" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>2</v>
       </c>
@@ -2157,10 +2304,13 @@
         <v>47</v>
       </c>
       <c r="Q16" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" ht="203" x14ac:dyDescent="0.35">
+        <v>324</v>
+      </c>
+      <c r="R16" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" ht="203" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>40</v>
       </c>
@@ -2201,8 +2351,14 @@
       <c r="P17" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" ht="87" x14ac:dyDescent="0.35">
+      <c r="Q17" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="R17" s="7" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" ht="87" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>12</v>
       </c>
@@ -2244,10 +2400,10 @@
         <v>47</v>
       </c>
       <c r="Q18" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>4</v>
       </c>
@@ -2288,8 +2444,11 @@
       <c r="P19" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+      <c r="Q19" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>1</v>
       </c>
@@ -2330,8 +2489,14 @@
       <c r="P20" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" ht="174" x14ac:dyDescent="0.35">
+      <c r="Q20" t="s">
+        <v>336</v>
+      </c>
+      <c r="R20" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>9</v>
       </c>
@@ -2372,8 +2537,11 @@
       <c r="P21" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="Q21" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>2</v>
       </c>
@@ -2422,8 +2590,14 @@
       <c r="P22" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+      <c r="Q22" t="s">
+        <v>341</v>
+      </c>
+      <c r="R22" s="7" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>1</v>
       </c>
@@ -2464,8 +2638,20 @@
       <c r="P23" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q23" t="s">
+        <v>343</v>
+      </c>
+      <c r="R23" s="7">
+        <v>29707</v>
+      </c>
+      <c r="S23" t="s">
+        <v>344</v>
+      </c>
+      <c r="T23" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>3</v>
       </c>
@@ -2511,10 +2697,10 @@
         <v>47</v>
       </c>
       <c r="Q24" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>2</v>
       </c>
@@ -2559,8 +2745,11 @@
       <c r="P25" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="Q25" s="5" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>1</v>
       </c>
@@ -2605,8 +2794,14 @@
       <c r="P26" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="Q26" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="R26" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>1</v>
       </c>
@@ -2655,8 +2850,14 @@
       <c r="P27" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="Q27" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="R27" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>2</v>
       </c>
@@ -2697,8 +2898,14 @@
       <c r="P28" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="29" spans="1:17" ht="116" x14ac:dyDescent="0.35">
+      <c r="Q28" t="s">
+        <v>347</v>
+      </c>
+      <c r="R28" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>1</v>
       </c>
@@ -2747,8 +2954,11 @@
       <c r="P29" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="30" spans="1:17" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="Q29" s="5" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>5</v>
       </c>
@@ -2797,7 +3007,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>5</v>
       </c>
@@ -2846,8 +3056,14 @@
       <c r="P31" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="32" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q31" s="10" t="s">
+        <v>348</v>
+      </c>
+      <c r="R31" s="7" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>2</v>
       </c>
@@ -2896,8 +3112,11 @@
       <c r="P32" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="33" spans="1:17" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="Q32" s="11" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>4</v>
       </c>
@@ -2940,8 +3159,11 @@
       <c r="P33" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="34" spans="1:17" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="Q33" s="11" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" ht="29" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>4</v>
       </c>
@@ -2982,8 +3204,11 @@
       <c r="P34" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="35" spans="1:17" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="Q34" s="11" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" ht="29" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>1</v>
       </c>
@@ -3030,7 +3255,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>1</v>
       </c>
@@ -3081,7 +3306,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>1</v>
       </c>
@@ -3132,7 +3357,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="38" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>1</v>
       </c>
@@ -3183,7 +3408,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="39" spans="1:17" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>1</v>
       </c>
@@ -3234,7 +3459,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="40" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>1</v>
       </c>
@@ -3285,7 +3510,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="87" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>1</v>
       </c>
@@ -3335,7 +3560,7 @@
         <v>47</v>
       </c>
       <c r="Q41" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="42" spans="1:17" ht="58" x14ac:dyDescent="0.35">
@@ -3440,7 +3665,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="44" spans="1:17" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>2</v>
       </c>
@@ -3492,11 +3717,14 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:Q44">
+  <sortState ref="A2:R44">
     <sortCondition ref="C1"/>
   </sortState>
+  <hyperlinks>
+    <hyperlink ref="Q6" r:id="rId1" display="https://www.mouser.de/ProductDetail/?qs=LLUE9lz1Ybc2beTd%252BaRHew%3D%3D"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="14" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="14" orientation="landscape" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
massenmail an trenz versendet mit allen samtec steckern als SMD
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents.xlsx
@@ -15,7 +15,7 @@
     <sheet name="BOM_UltraZOhm_CarrierBoard_4v00" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">BOM_UltraZOhm_CarrierBoard_4v00!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">BOM_UltraZOhm_CarrierBoard_4v00!$46:$46</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="354">
   <si>
     <t>Quantity</t>
   </si>
@@ -293,15 +293,6 @@
     <t>2.54mm Double Row Terminal Assembly, Right-Angled</t>
   </si>
   <si>
-    <t>2667420</t>
-  </si>
-  <si>
-    <t>200-IPL110201LDK</t>
-  </si>
-  <si>
-    <t>SAM10565-ND</t>
-  </si>
-  <si>
     <t>IPL1-103-01-L-D-K</t>
   </si>
   <si>
@@ -311,30 +302,12 @@
     <t>2.54mm Double Row Terminal Assembly</t>
   </si>
   <si>
-    <t>2856248</t>
-  </si>
-  <si>
-    <t>200-IPL110301LDK</t>
-  </si>
-  <si>
-    <t>SAM9594-ND</t>
-  </si>
-  <si>
     <t>IPL1-105-01-L-D-K</t>
   </si>
   <si>
     <t>X14</t>
   </si>
   <si>
-    <t>2308545</t>
-  </si>
-  <si>
-    <t>200-IPL110501LDK</t>
-  </si>
-  <si>
-    <t>SAM8825-ND</t>
-  </si>
-  <si>
     <t>IPL1-106-02-L-D-K</t>
   </si>
   <si>
@@ -353,15 +326,6 @@
     <t>X13</t>
   </si>
   <si>
-    <t>2856261</t>
-  </si>
-  <si>
-    <t>200-IPL110801LDK</t>
-  </si>
-  <si>
-    <t>SAM10585-ND</t>
-  </si>
-  <si>
     <t>IPL1-110-02-L-D-K</t>
   </si>
   <si>
@@ -608,15 +572,6 @@
     <t>2.54mm Single Row Terminal Assembly, Right Angle</t>
   </si>
   <si>
-    <t>2856253</t>
-  </si>
-  <si>
-    <t>200-IPL110401LSK</t>
-  </si>
-  <si>
-    <t>SAM9098-ND</t>
-  </si>
-  <si>
     <t>MAX14878</t>
   </si>
   <si>
@@ -989,9 +944,6 @@
     <t>Trenz?</t>
   </si>
   <si>
-    <t>alternative: UUJ2A221MNQ6MS (TE.DbLib/C_SMD)</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 28261 (Red) </t>
   </si>
   <si>
@@ -1004,12 +956,6 @@
     <t>0402 available</t>
   </si>
   <si>
-    <t xml:space="preserve"> bereits hinzugefügt - passst</t>
-  </si>
-  <si>
-    <t>alternative, nein, da 100V, evtl 100uF für 5V (C66), sonst hinzufügen</t>
-  </si>
-  <si>
     <t>hinzufügen oder 0402 auch ok</t>
   </si>
   <si>
@@ -1022,9 +968,6 @@
     <t>MBR0520L</t>
   </si>
   <si>
-    <t>hinzufügen, kleiner und günstigere alternative, ~100mA</t>
-  </si>
-  <si>
     <t xml:space="preserve">0603 ist Ok </t>
   </si>
   <si>
@@ -1086,13 +1029,73 @@
   </si>
   <si>
     <t>CDSOT23-T24CAN</t>
+  </si>
+  <si>
+    <t>done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done List </t>
+  </si>
+  <si>
+    <t>Trenz no 23116</t>
+  </si>
+  <si>
+    <t>ceramic caps 2x or 3x of 1206 Cs 6.3V</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Please Add</t>
+  </si>
+  <si>
+    <t>IPL1-104-02-L-S-K</t>
+  </si>
+  <si>
+    <t>IPL1-103-02-L-D-K</t>
+  </si>
+  <si>
+    <t>IPL1-108-02-L-D-K</t>
+  </si>
+  <si>
+    <t>IPL1-105-02-L-D-K</t>
+  </si>
+  <si>
+    <t>IPL1-102-02-L-D-K</t>
+  </si>
+  <si>
+    <t>Changed from THT to SMD</t>
+  </si>
+  <si>
+    <t>200-IPL110402LSK</t>
+  </si>
+  <si>
+    <t>200-IPL110302LDK</t>
+  </si>
+  <si>
+    <t>200-IPL110802LDK</t>
+  </si>
+  <si>
+    <t>200-IPL110502LDK</t>
+  </si>
+  <si>
+    <t>200-IPL110202LDK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">? Commercial grade? </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 24.11.2020 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email gesendet am: </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1104,6 +1107,22 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1171,7 +1190,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1192,14 +1211,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -1484,29 +1521,31 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T44"/>
+  <dimension ref="A1:T48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.1796875" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
     <col min="4" max="4" width="18.1796875" customWidth="1"/>
-    <col min="5" max="5" width="20.36328125" customWidth="1"/>
-    <col min="6" max="6" width="13.26953125" customWidth="1"/>
+    <col min="5" max="5" width="18.08984375" customWidth="1"/>
+    <col min="6" max="6" width="18.54296875" customWidth="1"/>
     <col min="7" max="7" width="45.36328125" customWidth="1"/>
     <col min="8" max="9" width="12.36328125" customWidth="1"/>
-    <col min="10" max="10" width="11" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="9.453125" customWidth="1"/>
-    <col min="13" max="13" width="8.36328125" customWidth="1"/>
-    <col min="14" max="14" width="7.26953125" customWidth="1"/>
-    <col min="15" max="15" width="9.90625" customWidth="1"/>
-    <col min="16" max="16" width="16" customWidth="1"/>
-    <col min="17" max="17" width="43.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.1796875" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" customWidth="1"/>
+    <col min="12" max="12" width="6" customWidth="1"/>
+    <col min="13" max="13" width="5.26953125" customWidth="1"/>
+    <col min="14" max="14" width="6.26953125" customWidth="1"/>
+    <col min="15" max="15" width="6.7265625" customWidth="1"/>
+    <col min="16" max="16" width="12.81640625" customWidth="1"/>
+    <col min="17" max="17" width="34.36328125" style="7" customWidth="1"/>
     <col min="18" max="18" width="26.6328125" style="7" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.26953125" style="7" customWidth="1"/>
+    <col min="20" max="20" width="10.90625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="1" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1555,138 +1594,146 @@
       <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
-        <v>319</v>
+      <c r="Q1" s="10" t="s">
+        <v>304</v>
       </c>
       <c r="R1" s="6"/>
-    </row>
-    <row r="2" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+    </row>
+    <row r="2" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>210</v>
+        <v>74</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>211</v>
+        <v>75</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>212</v>
+        <v>77</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>210</v>
+        <v>74</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>213</v>
+        <v>78</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="I2" s="3"/>
+        <v>79</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="J2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="N2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
+      <c r="O2" s="4" t="s">
+        <v>83</v>
+      </c>
       <c r="P2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q2" s="10" t="s">
-        <v>320</v>
-      </c>
-      <c r="R2" s="7" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q2" s="7" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>276</v>
+        <v>170</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>277</v>
+        <v>171</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>58</v>
+        <v>172</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>276</v>
+        <v>170</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>276</v>
+        <v>170</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>278</v>
+        <v>173</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>54</v>
+        <v>174</v>
       </c>
       <c r="J3" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>279</v>
+        <v>175</v>
       </c>
       <c r="L3" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>280</v>
+        <v>176</v>
       </c>
       <c r="N3" s="4" t="s">
         <v>36</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>281</v>
+        <v>177</v>
       </c>
       <c r="P3" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q3" s="10" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q3" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>155</v>
+        <v>39</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>156</v>
+        <v>190</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>155</v>
+        <v>191</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>155</v>
+        <v>39</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>158</v>
+        <v>193</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>54</v>
@@ -1695,51 +1742,43 @@
         <v>23</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="N4" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O4" s="4" t="s">
-        <v>161</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
       <c r="P4" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q4" s="10" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q4" s="11" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>256</v>
+        <v>139</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>257</v>
+        <v>140</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>256</v>
+        <v>141</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>256</v>
+        <v>139</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>258</v>
+        <v>52</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>158</v>
+        <v>53</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>54</v>
@@ -1748,172 +1787,148 @@
         <v>23</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="N5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>261</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
       <c r="P5" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q5" s="5" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" ht="58" x14ac:dyDescent="0.35">
+      <c r="Q5" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="R5" s="7" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>297</v>
+        <v>216</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>298</v>
+        <v>217</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>299</v>
+        <v>50</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>297</v>
+        <v>218</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>297</v>
+        <v>216</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>300</v>
+        <v>52</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>294</v>
+        <v>53</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>295</v>
+        <v>54</v>
       </c>
       <c r="J6" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>301</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="N6" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O6" s="4" t="s">
-        <v>303</v>
-      </c>
+        <v>219</v>
+      </c>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
       <c r="P6" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q6" s="8" t="s">
-        <v>328</v>
-      </c>
-      <c r="R6" s="7" t="s">
-        <v>329</v>
-      </c>
-      <c r="S6" s="9" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q6" s="11" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>1</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="N7" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O7" s="4" t="s">
-        <v>83</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
       <c r="P7" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q7" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="Q7" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>134</v>
+        <v>289</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>135</v>
+        <v>290</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>136</v>
+        <v>41</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>137</v>
+        <v>291</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>134</v>
+        <v>289</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>138</v>
+        <v>192</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>139</v>
+        <v>193</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>140</v>
+        <v>54</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>141</v>
+        <v>292</v>
       </c>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
@@ -1922,99 +1937,99 @@
       <c r="P8" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q8" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q8" s="7" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>2</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>184</v>
+        <v>76</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>186</v>
+        <v>165</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>186</v>
+        <v>166</v>
       </c>
       <c r="J9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="L9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="K9" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="L9" s="4" t="s">
-        <v>25</v>
-      </c>
       <c r="M9" s="4" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="N9" s="4" t="s">
         <v>36</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>189</v>
+        <v>169</v>
       </c>
       <c r="P9" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q9" t="s">
-        <v>352</v>
+      <c r="Q9" s="7" t="s">
+        <v>322</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>290</v>
+        <v>114</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>291</v>
+        <v>115</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>184</v>
+        <v>116</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>292</v>
+        <v>117</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>290</v>
+        <v>114</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>293</v>
+        <v>118</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>294</v>
+        <v>119</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>295</v>
+        <v>120</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>296</v>
+        <v>121</v>
       </c>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
@@ -2023,188 +2038,209 @@
       <c r="P10" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q10" s="10" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q10" s="11" t="s">
+        <v>324</v>
+      </c>
+      <c r="R10" s="7">
+        <v>29707</v>
+      </c>
+      <c r="S10" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="T10" s="7" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="4" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="Q11" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>162</v>
+        <v>64</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>163</v>
+        <v>65</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>162</v>
+        <v>67</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>162</v>
+        <v>64</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>164</v>
+        <v>68</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="I12" s="3"/>
+        <v>69</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>70</v>
+      </c>
       <c r="J12" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>166</v>
+        <v>71</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="N12" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O12" s="4" t="s">
-        <v>168</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
       <c r="P12" s="4" t="s">
         <v>47</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" ht="58" x14ac:dyDescent="0.35">
+        <v>328</v>
+      </c>
+      <c r="R12" s="7" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>1</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>39</v>
+        <v>130</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>40</v>
+        <v>131</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>41</v>
+        <v>106</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>42</v>
+        <v>132</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>39</v>
+        <v>130</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>43</v>
+        <v>133</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>44</v>
+        <v>134</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>45</v>
+        <v>135</v>
       </c>
       <c r="J13" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
+        <v>136</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>138</v>
+      </c>
       <c r="P13" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q13" s="10" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" ht="58" x14ac:dyDescent="0.35">
+      <c r="Q13" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>282</v>
+        <v>157</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>283</v>
+        <v>158</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>284</v>
+        <v>66</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>285</v>
+        <v>159</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>282</v>
+        <v>157</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>286</v>
+        <v>160</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>287</v>
+        <v>69</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>288</v>
+        <v>70</v>
       </c>
       <c r="J14" s="4" t="s">
         <v>25</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>289</v>
+        <v>161</v>
       </c>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
@@ -2213,322 +2249,281 @@
       <c r="P14" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q14" s="10" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" ht="58" x14ac:dyDescent="0.35">
+      <c r="Q14" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="R14" s="7" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>39</v>
+        <v>232</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>205</v>
+        <v>233</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>41</v>
+        <v>234</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>206</v>
+        <v>232</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>39</v>
+        <v>232</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>207</v>
+        <v>235</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>208</v>
+        <v>236</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>54</v>
+        <v>237</v>
       </c>
       <c r="J15" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="N15" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="K15" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
+      <c r="O15" s="4" t="s">
+        <v>240</v>
+      </c>
       <c r="P15" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q15" s="10" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="Q15" s="11" t="s">
+        <v>329</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>151</v>
+        <v>253</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>152</v>
+        <v>254</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>41</v>
+        <v>255</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>153</v>
+        <v>253</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>151</v>
+        <v>253</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>52</v>
+        <v>256</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>53</v>
+        <v>257</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>54</v>
+        <v>258</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
+        <v>259</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>260</v>
+      </c>
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
       <c r="P16" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q16" t="s">
-        <v>324</v>
-      </c>
-      <c r="R16" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" ht="203" x14ac:dyDescent="0.35">
-      <c r="A17" s="3">
-        <v>40</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>312</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>313</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>314</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>312</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>315</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>316</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="K17" s="4" t="s">
-        <v>318</v>
-      </c>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q17" s="10" t="s">
-        <v>337</v>
-      </c>
-      <c r="R17" s="7" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" ht="87" x14ac:dyDescent="0.35">
-      <c r="A18" s="3">
-        <v>12</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>309</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>311</v>
-      </c>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+      <c r="Q16" s="5" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A17" s="15"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="16"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
+      <c r="P17" s="16"/>
+      <c r="Q17" s="8"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A18" s="14" t="s">
+        <v>339</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>353</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>231</v>
+        <v>181</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>232</v>
+        <v>182</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>50</v>
+        <v>183</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>233</v>
+        <v>184</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>231</v>
+        <v>181</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>52</v>
+        <v>185</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>53</v>
+        <v>186</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="J19" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
+        <v>187</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>189</v>
+      </c>
       <c r="P19" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q19" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+      <c r="Q19" s="9" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>48</v>
+        <v>220</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>49</v>
+        <v>221</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>51</v>
+        <v>220</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>48</v>
+        <v>220</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>52</v>
+        <v>222</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>54</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="I20" s="3"/>
       <c r="J20" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
+        <v>224</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>225</v>
+      </c>
       <c r="N20" s="3"/>
       <c r="O20" s="3"/>
       <c r="P20" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q20" t="s">
-        <v>336</v>
-      </c>
-      <c r="R20" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" ht="58" x14ac:dyDescent="0.35">
+      <c r="Q20" s="9" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>304</v>
+        <v>226</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>305</v>
+        <v>227</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>41</v>
+        <v>106</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>306</v>
+        <v>226</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>304</v>
+        <v>226</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>207</v>
+        <v>228</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>54</v>
+        <v>230</v>
       </c>
       <c r="J21" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>307</v>
+        <v>231</v>
       </c>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
@@ -2537,1194 +2532,1250 @@
       <c r="P21" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q21" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q21" s="9" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>174</v>
+        <v>93</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>175</v>
+        <v>94</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>174</v>
+        <v>93</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>174</v>
+        <v>93</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>176</v>
+        <v>87</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>178</v>
-      </c>
+        <v>93</v>
+      </c>
+      <c r="I22" s="3"/>
       <c r="J22" s="4" t="s">
         <v>25</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>179</v>
+        <v>95</v>
       </c>
       <c r="L22" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="M22" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="N22" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O22" s="4" t="s">
-        <v>181</v>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
       <c r="P22" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q22" t="s">
-        <v>341</v>
-      </c>
-      <c r="R22" s="7" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+      <c r="Q22" s="5" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" ht="58" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>1</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>126</v>
+        <v>99</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>128</v>
+        <v>86</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>129</v>
+        <v>99</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>126</v>
+        <v>99</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>130</v>
+        <v>90</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="I23" s="4" t="s">
-        <v>132</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="I23" s="3"/>
       <c r="J23" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="N23" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="K23" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
-      <c r="O23" s="3"/>
+      <c r="O23" s="4" t="s">
+        <v>103</v>
+      </c>
       <c r="P23" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q23" t="s">
-        <v>343</v>
-      </c>
-      <c r="R23" s="7">
-        <v>29707</v>
-      </c>
-      <c r="S23" t="s">
-        <v>344</v>
-      </c>
-      <c r="T23" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q23" s="5" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" ht="58" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>224</v>
+        <v>340</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>225</v>
+        <v>179</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>224</v>
+        <v>340</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>224</v>
+        <v>340</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="J24" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="H24" s="4"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K24" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="L24" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="M24" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="N24" s="3"/>
-      <c r="O24" s="3"/>
-      <c r="P24" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="25" spans="1:20" ht="58" x14ac:dyDescent="0.35">
+      <c r="M24" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="R24" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="S24" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>28</v>
+        <v>341</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>31</v>
+        <v>341</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>28</v>
+        <v>341</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H25" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="I25" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="J25" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="H25" s="4"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K25" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="L25" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="M25" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="N25" s="3"/>
-      <c r="O25" s="3"/>
-      <c r="P25" s="4" t="s">
-        <v>38</v>
-      </c>
+      <c r="M25" t="s">
+        <v>347</v>
+      </c>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
       <c r="Q25" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="R25" s="7" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="26" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="S25" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>1</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>64</v>
+        <v>342</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>67</v>
+        <v>342</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>64</v>
+        <v>342</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="J26" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="H26" s="4"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K26" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="L26" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="M26" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="N26" s="3"/>
-      <c r="O26" s="3"/>
-      <c r="P26" s="4" t="s">
-        <v>47</v>
-      </c>
+      <c r="M26" t="s">
+        <v>348</v>
+      </c>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="4"/>
       <c r="Q26" s="5" t="s">
-        <v>347</v>
+        <v>307</v>
       </c>
       <c r="R26" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
+        <v>345</v>
+      </c>
+      <c r="S26" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>1</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>142</v>
+        <v>343</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>143</v>
+        <v>92</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>144</v>
+        <v>343</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>142</v>
+        <v>343</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="I27" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="J27" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K27" s="4" t="s">
-        <v>148</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="H27" s="4"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
       <c r="L27" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="M27" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="N27" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O27" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="P27" s="4" t="s">
-        <v>47</v>
-      </c>
+      <c r="M27" t="s">
+        <v>349</v>
+      </c>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="4"/>
       <c r="Q27" s="5" t="s">
-        <v>347</v>
+        <v>307</v>
       </c>
       <c r="R27" s="7" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="28" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+        <v>345</v>
+      </c>
+      <c r="S27" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>169</v>
+        <v>344</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>170</v>
+        <v>85</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>171</v>
+        <v>344</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>169</v>
+        <v>344</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="H28" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="I28" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="J28" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H28" s="4"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K28" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
-      <c r="O28" s="3"/>
-      <c r="P28" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>347</v>
+      <c r="M28" t="s">
+        <v>350</v>
+      </c>
+      <c r="N28" s="4"/>
+      <c r="O28" s="4"/>
+      <c r="P28" s="4"/>
+      <c r="Q28" s="5" t="s">
+        <v>307</v>
       </c>
       <c r="R28" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" ht="58" x14ac:dyDescent="0.35">
+        <v>345</v>
+      </c>
+      <c r="S28" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>116</v>
+        <v>202</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>117</v>
+        <v>203</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>119</v>
+        <v>202</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>116</v>
+        <v>202</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="I29" s="4" t="s">
-        <v>122</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="I29" s="3"/>
       <c r="J29" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>123</v>
+        <v>206</v>
       </c>
       <c r="L29" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>124</v>
+        <v>207</v>
       </c>
       <c r="N29" s="4" t="s">
         <v>36</v>
       </c>
       <c r="O29" s="4" t="s">
-        <v>125</v>
+        <v>208</v>
       </c>
       <c r="P29" s="4" t="s">
         <v>47</v>
       </c>
       <c r="Q29" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>5</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>270</v>
+        <v>86</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>271</v>
+        <v>204</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="I30" s="4" t="s">
-        <v>273</v>
-      </c>
+        <v>249</v>
+      </c>
+      <c r="I30" s="3"/>
       <c r="J30" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="L30" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K30" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="L30" s="4" t="s">
+      <c r="M30" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="N30" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="M30" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="N30" s="3"/>
-      <c r="O30" s="3"/>
+      <c r="O30" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="P30" s="4" t="s">
         <v>47</v>
       </c>
       <c r="Q30" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" ht="58" x14ac:dyDescent="0.35">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="87" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>247</v>
+        <v>104</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>248</v>
+        <v>105</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>249</v>
+        <v>106</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>247</v>
+        <v>107</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>247</v>
+        <v>104</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>250</v>
+        <v>108</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>251</v>
+        <v>109</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>252</v>
+        <v>110</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>253</v>
+        <v>111</v>
       </c>
       <c r="L31" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M31" s="4" t="s">
-        <v>254</v>
+        <v>112</v>
       </c>
       <c r="N31" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="O31" s="4" t="s">
-        <v>255</v>
+        <v>113</v>
       </c>
       <c r="P31" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q31" s="10" t="s">
-        <v>348</v>
-      </c>
-      <c r="R31" s="7" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q31" s="5" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>198</v>
+        <v>106</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>70</v>
+        <v>213</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="L32" s="4" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="M32" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="N32" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O32" s="4" t="s">
-        <v>204</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
       <c r="P32" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q32" s="11" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q32" s="7" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>235</v>
+        <v>16</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>236</v>
+        <v>17</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>235</v>
+        <v>19</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>235</v>
+        <v>16</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>237</v>
+        <v>20</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="I33" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="J33" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K33" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L33" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K33" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="L33" s="4" t="s">
-        <v>36</v>
-      </c>
       <c r="M33" s="4" t="s">
-        <v>240</v>
+        <v>26</v>
       </c>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
       <c r="P33" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q33" s="11" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+      <c r="Q33" s="5" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>241</v>
+        <v>150</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>242</v>
+        <v>151</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>118</v>
+        <v>58</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>241</v>
+        <v>150</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>241</v>
+        <v>150</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>243</v>
+        <v>152</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="I34" s="4" t="s">
-        <v>245</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="I34" s="3"/>
       <c r="J34" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K34" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
-      <c r="N34" s="3"/>
-      <c r="O34" s="3"/>
+        <v>154</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M34" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="N34" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="O34" s="4" t="s">
+        <v>156</v>
+      </c>
       <c r="P34" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q34" s="11" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+      <c r="Q34" s="5" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>102</v>
+        <v>241</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>103</v>
+        <v>242</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>102</v>
+        <v>241</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>102</v>
+        <v>241</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>87</v>
+        <v>243</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="I35" s="3"/>
+        <v>146</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>54</v>
+      </c>
       <c r="J35" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K35" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="L35" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K35" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="L35" s="4" t="s">
+      <c r="M35" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="N35" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="M35" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="N35" s="3"/>
-      <c r="O35" s="3"/>
+      <c r="O35" s="4" t="s">
+        <v>246</v>
+      </c>
       <c r="P35" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q35" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A36" s="3">
-        <v>1</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="H36" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="I36" s="3"/>
-      <c r="J36" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K36" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="L36" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M36" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="N36" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O36" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="P36" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q36" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A37" s="3">
-        <v>1</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="H37" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="I37" s="3"/>
-      <c r="J37" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K37" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="L37" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M37" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="N37" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O37" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="P37" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q37" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q35" s="8" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="B36" s="14"/>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A37" s="13" t="s">
+        <v>335</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>1</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>97</v>
+        <v>56</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>98</v>
+        <v>57</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>97</v>
+        <v>56</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>97</v>
+        <v>56</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>93</v>
+        <v>59</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="I38" s="3"/>
+        <v>56</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>60</v>
+      </c>
       <c r="J38" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>99</v>
+        <v>61</v>
       </c>
       <c r="L38" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M38" s="4" t="s">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="N38" s="4" t="s">
         <v>36</v>
       </c>
       <c r="O38" s="4" t="s">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="P38" s="4" t="s">
         <v>47</v>
       </c>
       <c r="Q38" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="39" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>84</v>
+        <v>261</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>85</v>
+        <v>262</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>84</v>
+        <v>261</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>84</v>
+        <v>261</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>87</v>
+        <v>263</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="I39" s="3"/>
+        <v>146</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>54</v>
+      </c>
       <c r="J39" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K39" s="4" t="s">
-        <v>88</v>
+        <v>264</v>
       </c>
       <c r="L39" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M39" s="4" t="s">
-        <v>89</v>
+        <v>265</v>
       </c>
       <c r="N39" s="4" t="s">
         <v>36</v>
       </c>
       <c r="O39" s="4" t="s">
-        <v>90</v>
+        <v>266</v>
       </c>
       <c r="P39" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q39" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q39" s="11" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>111</v>
+        <v>143</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>112</v>
+        <v>144</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>111</v>
+        <v>143</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>111</v>
+        <v>143</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="I40" s="3"/>
+        <v>146</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>54</v>
+      </c>
       <c r="J40" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K40" s="4" t="s">
-        <v>113</v>
+        <v>147</v>
       </c>
       <c r="L40" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M40" s="4" t="s">
-        <v>114</v>
+        <v>148</v>
       </c>
       <c r="N40" s="4" t="s">
         <v>36</v>
       </c>
       <c r="O40" s="4" t="s">
-        <v>115</v>
+        <v>149</v>
       </c>
       <c r="P40" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q40" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="41" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="Q40" s="11" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>1</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>56</v>
+        <v>122</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>57</v>
+        <v>123</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>58</v>
+        <v>124</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>56</v>
+        <v>125</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>56</v>
+        <v>122</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>59</v>
+        <v>126</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>56</v>
+        <v>127</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>60</v>
+        <v>128</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K41" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="L41" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M41" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="N41" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O41" s="4" t="s">
-        <v>63</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="L41" s="3"/>
+      <c r="M41" s="3"/>
+      <c r="N41" s="3"/>
+      <c r="O41" s="3"/>
       <c r="P41" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q41" s="5" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="42" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+      <c r="Q41" s="11" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>217</v>
+        <v>267</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>218</v>
+        <v>268</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>86</v>
+        <v>269</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>217</v>
+        <v>270</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>217</v>
+        <v>267</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>219</v>
+        <v>271</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="I42" s="3"/>
+        <v>272</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>273</v>
+      </c>
       <c r="J42" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K42" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="L42" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M42" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="N42" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O42" s="4" t="s">
-        <v>223</v>
-      </c>
+        <v>274</v>
+      </c>
+      <c r="L42" s="3"/>
+      <c r="M42" s="3"/>
+      <c r="N42" s="3"/>
+      <c r="O42" s="3"/>
       <c r="P42" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q42" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="43" spans="1:17" ht="58" x14ac:dyDescent="0.35">
+      <c r="Q42" s="11" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>86</v>
+        <v>172</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>219</v>
+        <v>278</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="I43" s="3"/>
+        <v>279</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>280</v>
+      </c>
       <c r="J43" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K43" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="L43" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M43" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="N43" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O43" s="4" t="s">
-        <v>267</v>
-      </c>
+        <v>281</v>
+      </c>
+      <c r="L43" s="3"/>
+      <c r="M43" s="3"/>
+      <c r="N43" s="3"/>
+      <c r="O43" s="3"/>
       <c r="P43" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q43" s="5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="44" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A44" s="3">
-        <v>2</v>
-      </c>
+      <c r="Q43" s="11" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="44" spans="1:20" ht="87" x14ac:dyDescent="0.35">
       <c r="B44" s="4" t="s">
-        <v>190</v>
+        <v>282</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>191</v>
+        <v>283</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>86</v>
+        <v>284</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>190</v>
+        <v>282</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>190</v>
+        <v>282</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>192</v>
+        <v>285</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="I44" s="3"/>
+        <v>279</v>
+      </c>
+      <c r="I44" s="4" t="s">
+        <v>280</v>
+      </c>
       <c r="J44" s="4" t="s">
         <v>23</v>
       </c>
       <c r="K44" s="4" t="s">
-        <v>193</v>
+        <v>286</v>
       </c>
       <c r="L44" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M44" s="4" t="s">
-        <v>194</v>
+        <v>287</v>
       </c>
       <c r="N44" s="4" t="s">
         <v>36</v>
       </c>
       <c r="O44" s="4" t="s">
-        <v>195</v>
+        <v>288</v>
       </c>
       <c r="P44" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q44" s="5" t="s">
-        <v>323</v>
+      <c r="Q44" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="R44" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="S44" s="8" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A45" s="3">
+        <v>1</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K45" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
+      <c r="N45" s="3"/>
+      <c r="O45" s="3"/>
+      <c r="P45" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q45" s="11" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="46" spans="1:20" s="1" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A46" s="3">
+        <v>3</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="I46" s="3"/>
+      <c r="J46" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K46" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="L46" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M46" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="N46" s="3"/>
+      <c r="O46" s="3"/>
+      <c r="P46" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q46" s="11" t="s">
+        <v>337</v>
+      </c>
+      <c r="R46" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="S46" s="7"/>
+      <c r="T46" s="7"/>
+    </row>
+    <row r="47" spans="1:20" ht="203" x14ac:dyDescent="0.35">
+      <c r="A47" s="3">
+        <v>40</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="J47" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K47" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
+      <c r="N47" s="3"/>
+      <c r="O47" s="3"/>
+      <c r="P47" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q47" s="11" t="s">
+        <v>318</v>
+      </c>
+      <c r="R47" s="7" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20" ht="87" x14ac:dyDescent="0.35">
+      <c r="A48" s="3">
+        <v>12</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J48" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K48" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
+      <c r="N48" s="3"/>
+      <c r="O48" s="3"/>
+      <c r="P48" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q48" s="7" t="s">
+        <v>321</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:R44">
+  <sortState ref="A1:T44">
     <sortCondition ref="C1"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="Q6" r:id="rId1" display="https://www.mouser.de/ProductDetail/?qs=LLUE9lz1Ybc2beTd%252BaRHew%3D%3D"/>
+    <hyperlink ref="Q44" r:id="rId1" display="https://www.mouser.de/ProductDetail/?qs=LLUE9lz1Ybc2beTd%252BaRHew%3D%3D"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="14" orientation="landscape" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="22" orientation="landscape" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated documentation of move to trenz lib, after discussion with simon and andreas on 17.12.2020
</commit_message>
<xml_diff>
--- a/Using Trenz Library/BOM_MissingComponents.xlsx
+++ b/Using Trenz Library/BOM_MissingComponents.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="360">
   <si>
     <t>Quantity</t>
   </si>
@@ -1113,11 +1113,26 @@
   <si>
     <t>check to replace with U23 - bitbucket issue opened</t>
   </si>
+  <si>
+    <t xml:space="preserve">replaced </t>
+  </si>
+  <si>
+    <t>simulated in lt-spice</t>
+  </si>
+  <si>
+    <t>compared and passed</t>
+  </si>
+  <si>
+    <t>calculated and passed</t>
+  </si>
+  <si>
+    <t>0402 used bc 0603 was not available</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1158,7 +1173,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1174,6 +1189,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1226,7 +1247,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1280,6 +1301,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -1300,7 +1327,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1697,6 +1724,9 @@
       <c r="Q2" s="7" t="s">
         <v>310</v>
       </c>
+      <c r="S2" s="21" t="s">
+        <v>356</v>
+      </c>
     </row>
     <row r="3" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
@@ -1752,6 +1782,9 @@
       </c>
       <c r="R3" s="18" t="s">
         <v>307</v>
+      </c>
+      <c r="S3" s="21" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
@@ -1801,6 +1834,9 @@
       <c r="R4" s="7" t="s">
         <v>300</v>
       </c>
+      <c r="S4" s="22" t="s">
+        <v>359</v>
+      </c>
     </row>
     <row r="5" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
@@ -1846,6 +1882,9 @@
       <c r="Q5" s="11" t="s">
         <v>300</v>
       </c>
+      <c r="S5" s="21" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="6" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
@@ -1894,6 +1933,9 @@
       <c r="R6" s="7" t="s">
         <v>300</v>
       </c>
+      <c r="S6" s="21" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="7" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
@@ -1950,6 +1992,9 @@
       <c r="R7" s="18" t="s">
         <v>307</v>
       </c>
+      <c r="S7" s="21" t="s">
+        <v>356</v>
+      </c>
     </row>
     <row r="8" spans="1:20" ht="87" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
@@ -2005,6 +2050,9 @@
       </c>
       <c r="R8" s="18" t="s">
         <v>354</v>
+      </c>
+      <c r="S8" s="21" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.35">

</xml_diff>